<commit_message>
9/3 美股版23:00盘中监控: 🟢恐慌解除(纳指29420>MA5 29306)实盘重建7只持仓8,011(NEM/NOW/HOOD/SPCX/NFLX/LITE/MU), ZS被MU挤出; 空仓3日后恢复建仓
</commit_message>
<xml_diff>
--- a/backtest/results_us100/七星美股版_实盘交易记录.xlsx
+++ b/backtest/results_us100/七星美股版_实盘交易记录.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="50">
   <si>
     <t>交易日期</t>
   </si>
@@ -76,6 +76,9 @@
     <t>2026-09-02</t>
   </si>
   <si>
+    <t>2026-09-03</t>
+  </si>
+  <si>
     <t>EOG</t>
   </si>
   <si>
@@ -118,6 +121,9 @@
     <t>HOOD</t>
   </si>
   <si>
+    <t>MU</t>
+  </si>
+  <si>
     <t>买入</t>
   </si>
   <si>
@@ -155,6 +161,9 @@
   </si>
   <si>
     <t>NDX5恐慌空仓</t>
+  </si>
+  <si>
+    <t>持久化: 排名2</t>
   </si>
 </sst>
 </file>
@@ -512,7 +521,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -546,13 +555,13 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E2">
         <v>143.76</v>
@@ -564,7 +573,7 @@
         <v>1.850703026003797</v>
       </c>
       <c r="H2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -572,13 +581,13 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E3">
         <v>296.92</v>
@@ -590,7 +599,7 @@
         <v>1.048568944225358</v>
       </c>
       <c r="H3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -598,13 +607,13 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E4">
         <v>174.77</v>
@@ -616,7 +625,7 @@
         <v>0.5049917097513827</v>
       </c>
       <c r="H4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -624,13 +633,13 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E5">
         <v>170.94</v>
@@ -642,7 +651,7 @@
         <v>0.5049917097513827</v>
       </c>
       <c r="H5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -650,13 +659,13 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E6">
         <v>140.52</v>
@@ -668,7 +677,7 @@
         <v>1.850703026003797</v>
       </c>
       <c r="H6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -676,13 +685,13 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E7">
         <v>175.36</v>
@@ -694,7 +703,7 @@
         <v>1.290286230231872</v>
       </c>
       <c r="H7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -702,13 +711,13 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E8">
         <v>126.13</v>
@@ -720,7 +729,7 @@
         <v>0.8744027938204831</v>
       </c>
       <c r="H8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -728,13 +737,13 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E9">
         <v>115.71</v>
@@ -746,7 +755,7 @@
         <v>0.5494489168637116</v>
       </c>
       <c r="H9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -754,13 +763,13 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E10">
         <v>392.73</v>
@@ -772,7 +781,7 @@
         <v>0.5675635282792316</v>
       </c>
       <c r="H10" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -780,13 +789,13 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E11">
         <v>46.48</v>
@@ -798,7 +807,7 @@
         <v>8.156762029709951</v>
       </c>
       <c r="H11" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -806,13 +815,13 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E12">
         <v>146.89</v>
@@ -824,7 +833,7 @@
         <v>6.871727331450243</v>
       </c>
       <c r="H12" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -832,13 +841,13 @@
         <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C13" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D13" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E13">
         <v>357.14</v>
@@ -850,7 +859,7 @@
         <v>0.5675635282792316</v>
       </c>
       <c r="H13" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -858,13 +867,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E14">
         <v>838.28</v>
@@ -876,7 +885,7 @@
         <v>4.291107478203252</v>
       </c>
       <c r="H14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -884,13 +893,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C15" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D15" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E15">
         <v>286</v>
@@ -902,7 +911,7 @@
         <v>1.048568944225358</v>
       </c>
       <c r="H15" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -910,13 +919,13 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C16" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D16" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E16">
         <v>73.09999999999999</v>
@@ -928,7 +937,7 @@
         <v>4.490398840085638</v>
       </c>
       <c r="H16" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -936,13 +945,13 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C17" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D17" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E17">
         <v>69.37</v>
@@ -954,7 +963,7 @@
         <v>4.490398840085638</v>
       </c>
       <c r="H17" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -962,13 +971,13 @@
         <v>15</v>
       </c>
       <c r="B18" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C18" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D18" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E18">
         <v>135.76</v>
@@ -980,7 +989,7 @@
         <v>7.677801960298933</v>
       </c>
       <c r="H18" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -988,13 +997,13 @@
         <v>16</v>
       </c>
       <c r="B19" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C19" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D19" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E19">
         <v>908.0599999999999</v>
@@ -1006,7 +1015,7 @@
         <v>4.291107478203252</v>
       </c>
       <c r="H19" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1014,13 +1023,13 @@
         <v>16</v>
       </c>
       <c r="B20" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C20" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D20" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E20">
         <v>81.91</v>
@@ -1032,7 +1041,7 @@
         <v>3.650597275283464</v>
       </c>
       <c r="H20" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1040,13 +1049,13 @@
         <v>17</v>
       </c>
       <c r="B21" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C21" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D21" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E21">
         <v>152.61</v>
@@ -1058,7 +1067,7 @@
         <v>6.871727331450243</v>
       </c>
       <c r="H21" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1066,13 +1075,13 @@
         <v>17</v>
       </c>
       <c r="B22" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C22" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D22" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E22">
         <v>917.05</v>
@@ -1084,7 +1093,7 @@
         <v>4.101054724283061</v>
       </c>
       <c r="H22" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1092,13 +1101,13 @@
         <v>18</v>
       </c>
       <c r="B23" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C23" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D23" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E23">
         <v>39.66</v>
@@ -1110,7 +1119,7 @@
         <v>8.156762029709951</v>
       </c>
       <c r="H23" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1118,13 +1127,13 @@
         <v>18</v>
       </c>
       <c r="B24" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C24" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D24" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E24">
         <v>102.89</v>
@@ -1136,7 +1145,7 @@
         <v>4.548675345807821</v>
       </c>
       <c r="H24" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1144,13 +1153,13 @@
         <v>19</v>
       </c>
       <c r="B25" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C25" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D25" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E25">
         <v>176.29</v>
@@ -1162,7 +1171,7 @@
         <v>1.290286230231872</v>
       </c>
       <c r="H25" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1170,13 +1179,13 @@
         <v>19</v>
       </c>
       <c r="B26" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C26" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D26" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E26">
         <v>139.32</v>
@@ -1188,7 +1197,7 @@
         <v>0.8744027938204831</v>
       </c>
       <c r="H26" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -1196,13 +1205,13 @@
         <v>19</v>
       </c>
       <c r="B27" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C27" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D27" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E27">
         <v>125.76</v>
@@ -1214,7 +1223,7 @@
         <v>0.5494489168637116</v>
       </c>
       <c r="H27" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -1222,13 +1231,13 @@
         <v>19</v>
       </c>
       <c r="B28" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C28" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D28" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E28">
         <v>140.45</v>
@@ -1240,7 +1249,7 @@
         <v>7.677801960298933</v>
       </c>
       <c r="H28" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1248,13 +1257,13 @@
         <v>19</v>
       </c>
       <c r="B29" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C29" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D29" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E29">
         <v>82.61</v>
@@ -1266,7 +1275,7 @@
         <v>3.650597275283464</v>
       </c>
       <c r="H29" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -1274,13 +1283,13 @@
         <v>19</v>
       </c>
       <c r="B30" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C30" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D30" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E30">
         <v>860</v>
@@ -1292,7 +1301,7 @@
         <v>4.101054724283061</v>
       </c>
       <c r="H30" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -1300,13 +1309,13 @@
         <v>19</v>
       </c>
       <c r="B31" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C31" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D31" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E31">
         <v>106.97</v>
@@ -1318,6 +1327,188 @@
         <v>4.548675345807821</v>
       </c>
       <c r="H31" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
+      <c r="A32" t="s">
+        <v>20</v>
+      </c>
+      <c r="B32" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32" t="s">
+        <v>36</v>
+      </c>
+      <c r="E32">
+        <v>129.35</v>
+      </c>
+      <c r="F32">
+        <v>54</v>
+      </c>
+      <c r="G32">
+        <v>13.60666220243627</v>
+      </c>
+      <c r="H32" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
+      <c r="A33" t="s">
+        <v>20</v>
+      </c>
+      <c r="B33" t="s">
+        <v>25</v>
+      </c>
+      <c r="C33" t="s">
+        <v>25</v>
+      </c>
+      <c r="D33" t="s">
+        <v>36</v>
+      </c>
+      <c r="E33">
+        <v>144.25</v>
+      </c>
+      <c r="F33">
+        <v>48</v>
+      </c>
+      <c r="G33">
+        <v>6.582518255184114</v>
+      </c>
+      <c r="H33" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34" t="s">
+        <v>20</v>
+      </c>
+      <c r="B34" t="s">
+        <v>34</v>
+      </c>
+      <c r="C34" t="s">
+        <v>34</v>
+      </c>
+      <c r="D34" t="s">
+        <v>36</v>
+      </c>
+      <c r="E34">
+        <v>123.23</v>
+      </c>
+      <c r="F34">
+        <v>56</v>
+      </c>
+      <c r="G34">
+        <v>5.712362312360674</v>
+      </c>
+      <c r="H34" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
+      <c r="A35" t="s">
+        <v>20</v>
+      </c>
+      <c r="B35" t="s">
+        <v>32</v>
+      </c>
+      <c r="C35" t="s">
+        <v>32</v>
+      </c>
+      <c r="D35" t="s">
+        <v>36</v>
+      </c>
+      <c r="E35">
+        <v>148.95</v>
+      </c>
+      <c r="F35">
+        <v>46</v>
+      </c>
+      <c r="G35">
+        <v>3.492246342195308</v>
+      </c>
+      <c r="H35" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36" t="s">
+        <v>20</v>
+      </c>
+      <c r="B36" t="s">
+        <v>33</v>
+      </c>
+      <c r="C36" t="s">
+        <v>33</v>
+      </c>
+      <c r="D36" t="s">
+        <v>36</v>
+      </c>
+      <c r="E36">
+        <v>82.47</v>
+      </c>
+      <c r="F36">
+        <v>84</v>
+      </c>
+      <c r="G36">
+        <v>2.542131667306065</v>
+      </c>
+      <c r="H36" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37" t="s">
+        <v>20</v>
+      </c>
+      <c r="B37" t="s">
+        <v>30</v>
+      </c>
+      <c r="C37" t="s">
+        <v>30</v>
+      </c>
+      <c r="D37" t="s">
+        <v>36</v>
+      </c>
+      <c r="E37">
+        <v>849.61</v>
+      </c>
+      <c r="F37">
+        <v>8</v>
+      </c>
+      <c r="G37">
+        <v>1.638536449057692</v>
+      </c>
+      <c r="H37" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" t="s">
+        <v>20</v>
+      </c>
+      <c r="B38" t="s">
+        <v>35</v>
+      </c>
+      <c r="C38" t="s">
+        <v>35</v>
+      </c>
+      <c r="D38" t="s">
+        <v>36</v>
+      </c>
+      <c r="E38">
+        <v>946.45</v>
+      </c>
+      <c r="F38">
+        <v>7</v>
+      </c>
+      <c r="G38">
+        <v>1.104587343460544</v>
+      </c>
+      <c r="H38" t="s">
         <v>46</v>
       </c>
     </row>

</xml_diff>